<commit_message>
chore: archive legacy agents/skills/commands, update mapa and agent docs
- Move 18 legacy agents, 10 eng-* commands, and 39 legacy skills to archive/
- Update docs/usage/agents.md with individual agent role descriptions
- Update mapa_operacional.xlsx with OpenTrust runtime entries
- Fix tests referencing archived legacy files (use active opentrust-* skills)
</commit_message>
<xml_diff>
--- a/mapa_operacional.xlsx
+++ b/mapa_operacional.xlsx
@@ -867,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1347,6 +1347,318 @@
       <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Parallel agent work requiring file isolation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OTF01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>opentrust-explore</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Read-only exploration: inspect current state, identify scope, risks, and needed selectors</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>read-only</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Inspect &gt; identify scope &gt; assess risk &gt; propose selectors</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK07</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>OTLD01; OTLD02; OTLD03; OTLD09</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>global/commands/ot-explore.md</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Phase 1 — before any work begins</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OTF02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>opentrust-propose</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Produce approved task contract with acceptance criteria, test plan, and retrieval selectors</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>read-only</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Write proposal &gt; compare alternatives &gt; define AC &gt; list selectors &gt; approval gate</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK03</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>OTLD01; OTLD02; OTLD03; OTLD09</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>global/commands/ot-propose.md</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Phase 2 — after Explore, before implementation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OTF03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>opentrust-apply</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Implement approved task contract with TDD-First for behavioral changes</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>sequential</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Create task plan &gt; TDD RED &gt; implement &gt; TDD GREEN &gt; validate &gt; update plan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>OTSK02; OTSK03</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>OTLD04; OTLD05; OTAG11; OTAG12</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>global/commands/ot-apply.md</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Phase 3 — implementation microincrements</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OTF04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Independent review of diff, tests, security, architecture, and docs</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>read-only</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Read diff &gt; verify AC &gt; run tests &gt; check security &gt; review docs &gt; approve/block</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>OTSK04</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>OTLD06; OTAG19; OTAG20; OTAG21</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>global/commands/ot-review.md</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Phase 4 — pre-delivery quality gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OTF05</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>opentrust-ship</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Prepare commit, push, and PR using Conventional Commits</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Archive &gt; commit &gt; push &gt; PR &gt; tag &gt; release</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>OTSK05; OTSK06</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>OTLD08; OTAG25; OTAG26</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>global/commands/ot-ship.md</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Phase 5 — final delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OTF06</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>opentrust-incident</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Triage incidents with smallest safe containment and recovery steps</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>sequential</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Diagnose &gt; contain &gt; recover &gt; validate &gt; report</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>OTSK06</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>OTLD07; OTAG24</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>global/commands/ot-incident.md</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Incident response — any phase</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1903,6 +2215,230 @@
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Any time to check progress or orientation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OTC01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ot-explore</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Perform read-only exploration: inspect current state, identify scope, files, risks, and needed Retrieval Context selectors</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>global/commands/ot-explore.md</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Phase 1 — before any work begins, to understand current state and scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OTC02</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ot-propose</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Produce task contract with acceptance criteria, test plan, and Retrieval Context selectors</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>global/commands/ot-propose.md</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Phase 2 — after Explore, to formalize scope and get approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OTC03</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ot-apply</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Implement only an approved task contract with TDD-First for behavioral changes</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>global/commands/ot-apply.md</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Phase 3 — after proposal approval, to implement one microincrement at a time</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OTC04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ot-review</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Independent review of implementation diff, validation evidence, tests, security, architecture, and docs</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>global/commands/ot-review.md</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Phase 4 — after Apply, before delivery, for independent quality gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OTC05</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ot-ship</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Prepare commit, PR, and release artifacts only when explicitly requested. Uses Conventional Commits in English.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>global/commands/ot-ship.md</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Phase 5 — after Review approval, for final delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>OTC06</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ot-status</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Summarize current state: branch, diff, active task, pending validation, and next step</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>global/commands/ot-status.md</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Any phase — for status reporting and context resumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>OTC07</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ot-incident</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Diagnose incident or failure, collect evidence, propose fix, validate resolution</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>global/commands/ot-incident.md</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>When a runtime, test, build, deployment, or configuration incident occurs</t>
         </is>
       </c>
     </row>
@@ -44516,7 +45052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W32"/>
+  <dimension ref="A1:W39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.83203125" customWidth="1" min="1" max="1"/>
@@ -48043,6 +48579,629 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>OTSK01</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Create or refine task contracts using TASK_CONTRACT.md template including Retrieval Context selectors</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>When a task needs formal scope, acceptance criteria, retrieval requirements, and delivery rules before implementation</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>task request; scope description; user intent</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>task contract with acceptance criteria, retrieval selectors, teams involved</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>global/skills/opentrust-task-contract/SKILL.md</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Contract must reference approved selectors; no raw chunks in output</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Must include Retrieval Context section</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>OTLD01; OTLD02; OTLD03; OTLD04; OTLD08</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>OTSK02; OTSK03; OTSK05</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>opentrust; workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>OTSK02</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Enforce test-first workflow when behavior or rules change — define failing test, implement, validate</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>When changing executable behavior (bugfix, new feature, refactoring of behavior)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>behavior description; acceptance criteria; existing test files</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>RED evidence; GREEN evidence; refactored code; test results</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>global/skills/opentrust-tdd/SKILL.md</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Must show RED before implementation; GREEN must verify behavior</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Not for documentation-only changes</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>OTLD04; OTLD05; OTAG11; OTAG16</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK03</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>opentrust; workflow; tdd</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>OTSK03</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>opentrust-spec-change</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Guide structured spec and design changes using Explore -&gt; Propose before Apply</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>When a feature or change requires formal specification, business rule analysis, impact assessment, or an approved plan before code</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>change request; context; affected boundaries</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>spec document; task plan; approved plan with AC</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>global/skills/opentrust-spec-change/SKILL.md</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Spec must include AC, scope, risks, and retrieval selectors</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Not for trivial or fully-scoped tasks</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>sdd; OTLD02; OTLD03; OTLD04</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK02</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>opentrust; workflow; spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>OTSK04</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Review diff, tests, security, architecture, and docs — approve or block with evidence</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>When a diff is ready for independent review before delivery</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>diff; implementation plan; test results; AC</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>review report with findings, blocking issues, or approval</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>global/skills/opentrust-review/SKILL.md</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Must verify AC, scope, security, edge cases, tests, and docs</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Not for trivial formatting-only changes</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>OTLD06; OTAG19</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK02</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>opentrust; workflow; review</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>OTSK05</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>opentrust-delivery</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Prepare commit, push, and pull request using Conventional Commits in English. Avoid unrelated files.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>When approved work is ready for version control and delivery</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>approved scope; diff; validation evidence</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>commit; push; PR (when requested)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>global/skills/opentrust-delivery/SKILL.md</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Only deliver approved scope; never include unrelated files</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Not for unapproved changes</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>OTLD08; OTAG25</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>OTSK04; OTSK06</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>opentrust; workflow; delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>OTSK06</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>opentrust-observability</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Require execution reports, validation evidence, and operational notes. Do not implement external telemetry yet.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>When work requires traceability, decision logging, or deployment evidence</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>phase; task; decisions made</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>execution report with validation evidence and operational notes</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>global/skills/opentrust-observability/SKILL.md</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Must log decisions, evidence, blockers, and next actions</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Not for external telemetry or monitoring infrastructure</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>OTLD01; OTLD07; OTAG23</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK04</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>opentrust; workflow; observability</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>OTSK07</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>opentrust-reference-research</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Use Operational Retrieval Map selectors. Request synthesis only. No raw chunks in output or commits.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>When domain knowledge, architecture patterns, or reference material is needed during any workflow phase</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>selector query (CTX/SK/B/DOC); task contract</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>synthesized response with source IDs; no raw chunks</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>global/skills/opentrust-reference-research/SKILL.md</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Must cite source IDs; no raw chunks in versioned output</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Not for trivial or fully-scoped tasks</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>OTLD09; OTAG28; OTAG27</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK03</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>opentrust; workflow; retrieval</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -48054,7 +49213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y18"/>
+  <dimension ref="A1:Y56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.83203125" customWidth="1" min="1" max="1"/>
@@ -50265,6 +51424,3018 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>OTLD01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>trust-lead</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Coordinates cross-team communication, decision logging, meeting facilitation, and process health</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Phase 1-2 (Explore/Propose), cross-team coordination, workflow governance</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Coordinate OpenTrust workflow, decisions, handoffs, and process health</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract; opentrust-observability; opentrust-review</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>global/agents/trust-lead.md</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract; opentrust-observability</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>coordination-facilitator; meeting-scribe; decision-logger</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>OpenTrust team lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>OTLD02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>product-lead</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Product strategy, discovery, requirements, acceptance criteria, and story slicing</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Phase 1-2 (Explore/Propose), requirements gathering, scope definition</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Turn vague requests into actionable, testable scope</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract; opentrust-spec-change</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>global/agents/product-lead.md</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract; opentrust-spec-change</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>product-discovery; requirements-analyzer; story-slicer</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>OpenTrust team lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>OTLD03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>architecture-lead</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Structural decisions, domain modeling, API/database contracts, distributed systems, and ADRs</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Phase 2-3 (Propose/Apply), architecture decisions, trade-off analysis</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Guide structural decisions and trade-offs</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>opentrust-spec-change; opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>global/agents/architecture-lead.md</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>opentrust-spec-change; opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>architecture-decision-designer; domain-modeler; api-database-designer; distributed-systems-reviewer</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>OpenTrust team lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>OTLD04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>engineering-lead</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Implementation, refactoring, performance, security, and privacy leadership</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Phase 3 (Apply), implementation, code changes within approved scope</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Coordinate implementation work inside approved scope</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>opentrust-tdd; opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>global/agents/engineering-lead.md</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>opentrust-tdd; opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>feature-implementer; code-refactoring-specialist; performance-engineer; security-reviewer; privacy-reviewer</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>OpenTrust team lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>OTLD05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>quality-lead</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Test strategy, TDD, integration tests, end-to-end tests, and quality gates</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Phase 3-4 (Apply/Review), test planning, quality verification</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Define and verify quality strategy</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>opentrust-tdd; opentrust-review</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>global/agents/quality-lead.md</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>opentrust-tdd; opentrust-review</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>tdd-engineer; integration-tester; testing-strategy-designer</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>OpenTrust team lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>OTLD06</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>review-lead</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Independent review, compliance, UX/accessibility review, and delivery gating</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Phase 4 (Review), pre-delivery quality gate, compliance check</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Gate changes through independent review</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>global/agents/review-lead.md</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>code-reviewer; compliance-auditor; ux-accessibility-reviewer</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>OpenTrust team lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>OTLD07</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>devops-lead</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CI/CD, infrastructure, observability, and incident response leadership</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Any phase, infrastructure/ops decisions, incident triage</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Coordinate delivery infrastructure and operational reliability</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>opentrust-observability; opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>global/agents/devops-lead.md</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>opentrust-observability; opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>ci-cd-infrastructure-engineer; observability-designer; incident-triage-specialist</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>OpenTrust team lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>OTLD08</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>delivery-lead</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Release management, versioning, changelog, and deployment coordination</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Phase 5 (Ship), post-review release preparation</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Prepare approved work for release</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>opentrust-delivery; opentrust-observability</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>global/agents/delivery-lead.md</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>opentrust-delivery; opentrust-observability</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>release-manager; changelog-writer</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>OpenTrust team lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>OTLD09</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>knowledge-lead</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Context retrieval, reference library management, documentation generation, and skill creation</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>All phases, when retrieval or reference material is needed</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Provide selector-based synthesis and reference governance. Only team that calls the retrieval provider directly.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>opentrust-reference-research; opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>global/agents/knowledge-lead.md</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>opentrust-reference-research; opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>context-historian; reference-librarian; documentation-skill-creator</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>OpenTrust team lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>OTAG01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>coordination-facilitator</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Facilitates Trust Coordination handoffs, meetings, and cross-team alignment</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Phase 1-2, cross-team coordination, blocker resolution</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Facilitate cross-team coordination, handoffs, and blocker alignment</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>global/agents/coordination-facilitator.md</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>trust-lead</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>OTAG02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>meeting-scribe</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Captures meeting notes, action items, and handoff evidence for Trust Coordination</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>After meetings, handoffs, decision points</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Capture concise meeting notes, action items, open questions, and evidence</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>opentrust-observability</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>global/agents/meeting-scribe.md</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>opentrust-observability</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>trust-lead</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>OTAG03</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>decision-logger</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Records decisions, rationale, and unresolved risks for Trust Coordination</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>After decisions, trade-off evaluations, blocked tasks</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Record decisions, rationale, alternatives rejected, risks, and follow-up needs</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>opentrust-observability</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>global/agents/decision-logger.md</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>opentrust-observability</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>trust-lead</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>OTAG04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>product-discovery</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Explores product problems, users, outcomes, and discovery risks</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Phase 1 (Explore), before shaping any product work</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Clarify product problem, users, outcomes, assumptions, risks, and discovery questions</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>global/agents/product-discovery.md</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>product-lead</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>OTAG05</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>requirements-analyzer</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Analyzes requirements, constraints, acceptance criteria, and gaps</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Phase 2 (Propose), requirements refinement</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Analyze requirements, constraints, dependencies, acceptance criteria, and missing details</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>global/agents/requirements-analyzer.md</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>product-lead</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>OTAG06</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>story-slicer</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Slices product work into small testable stories with explicit exclusions</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Phase 2 (Propose), after requirements are clear</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Slice scoped work into small testable stories, edges, and explicit out-of-scope items</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract; opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>global/agents/story-slicer.md</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract; opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>product-lead</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>OTAG07</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>architecture-decision-designer</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Compares architecture options, trade-offs, and ADR-ready decisions</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Phase 2-3 (Propose/Apply), architecture decisions</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Compare architecture options, constraints, trade-offs, and ADR-ready decision points</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>opentrust-spec-change</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>global/agents/architecture-decision-designer.md</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>opentrust-spec-change</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>architecture-lead</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>OTAG08</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>domain-modeler</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Shapes domain models, concepts, boundaries, and core language</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Phase 2-3 (Propose/Apply), domain modeling</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Define domain concepts, boundaries, relationships, invariants, and shared language</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>opentrust-spec-change</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>global/agents/domain-modeler.md</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>opentrust-spec-change</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>architecture-lead</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>OTAG09</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>api-database-designer</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Designs APIs, schemas, data contracts, and evolution paths</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Phase 3 (Apply), API/database design</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Design APIs, schemas, data models, contracts, evolution, and migration paths</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>opentrust-spec-change</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>global/agents/api-database-designer.md</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>opentrust-spec-change</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>architecture-lead</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>OTAG10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>distributed-systems-reviewer</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Reviews distributed-systems patterns, consistency, trade-offs, and failure modes</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Phase 4 (Review), distributed systems audit</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Review consistency, concurrency, failures, retries, eventual consistency, and trade-offs</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>global/agents/distributed-systems-reviewer.md</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>architecture-lead</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>OTAG11</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>feature-implementer</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Build approved feature changes in small validated increments</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Phase 3 (Apply), feature implementation</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Implements approved changes. Keeps diff small. Runs focused validation.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>global/agents/feature-implementer.md</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>engineering-lead</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>OTAG12</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>code-refactoring-specialist</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Refactor code incrementally while preserving approved behavior</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Phase 3 (Apply), refactoring tasks</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Improves structure with behavior preserved. Prefers smallest safe change.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>global/agents/code-refactoring-specialist.md</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>engineering-lead</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>OTAG13</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>performance-engineer</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Find and reduce performance bottlenecks with measured evidence</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Phase 3-4 (Apply/Review), performance optimization</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Profiles hot paths. Suggests smallest fix with evidence.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>opentrust-tdd; opentrust-review</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>global/agents/performance-engineer.md</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>opentrust-tdd; opentrust-review</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>engineering-lead</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>OTAG14</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>security-reviewer</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Review implementation for security risks and minimum effective controls</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Phase 4 (Review), security audit</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Checks auth, secrets, trust boundaries, unsafe defaults, dependency risk</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>global/agents/security-reviewer.md</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>engineering-lead</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr"/>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>OTAG15</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>privacy-reviewer</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Review privacy impact, data handling, retention, and exposure risks</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Phase 4 (Review), privacy audit</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Checks data minimization, consent, retention, sharing, logging exposure</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>global/agents/privacy-reviewer.md</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>engineering-lead</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr"/>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>OTAG16</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>tdd-engineer</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Drive red-green-refactor for smallest useful automated tests</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Phase 3 (Apply), test-first for behavioral changes</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Defines failing test first. Confirms red and green evidence.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>global/agents/tdd-engineer.md</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>quality-lead</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>OTAG17</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>integration-tester</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Verify integrated behavior across boundaries with focused evidence</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Phase 4 (Review), integration test verification</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Checks behavior across modules, contracts, fixtures, and regressions</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>opentrust-tdd; opentrust-review</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>global/agents/integration-tester.md</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>opentrust-tdd; opentrust-review</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>quality-lead</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>OTAG18</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>testing-strategy-designer</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Design lean test strategy matched to risk, scope, and feedback speed</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Phase 2-3 (Propose/Apply), test strategy definition</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Chooses test levels, coverage targets, and smallest useful checks</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract; opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>global/agents/testing-strategy-designer.md</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>opentrust-task-contract; opentrust-tdd</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>quality-lead</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>OTAG19</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>code-reviewer</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Read-only independent review of implementation diff, tests, scope, security, contracts, migrations, dependencies, and regressions before delivery</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Phase 4 (Review), pre-delivery code review</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Read-only code review. Checks correctness, scope compliance, security, privacy, contracts, dependencies, legacy preservation, error paths, docs.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>global/agents/code-reviewer.md</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>review-lead</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>Preserved legacy agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>OTAG20</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>compliance-auditor</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Auditar conformidade — dependencias, licencas, vulnerabilidades, supply chain, regulamentacao e politicas</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Phase 4 (Review), compliance/security audit</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Dependency audit, license checks, vulnerability scanning, supply chain verification, regulatory compliance</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>global/agents/compliance-auditor.md</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>review-lead</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>Preserved legacy agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>OTAG21</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ux-accessibility-reviewer</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Review user experience and accessibility issues before delivery gates</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Phase 4 (Review), UX/accessibility audit</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Checks flows, clarity, keyboard access, semantics, and blocking UX risks</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>global/agents/ux-accessibility-reviewer.md</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>opentrust-review</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>review-lead</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr"/>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>OTAG22</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ci-cd-infrastructure-engineer</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Designs CI/CD flow, pipeline guards, and infrastructure delivery checks</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Phase 3-5 (Apply to Ship), CI/CD/infra decisions</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Shapes CI/CD and infra rollout plan. Checks pipeline gates, rollback path, and deploy safety.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>opentrust-observability; opentrust-delivery</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>global/agents/ci-cd-infrastructure-engineer.md</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>opentrust-observability; opentrust-delivery</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>devops-lead</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr"/>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>OTAG23</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>observability-designer</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Designs logs, metrics, traces, alerts, and debug paths</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Phase 3-5 (Apply to Ship), observability definition</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Defines observability plan for logs, metrics, traces, and alerts.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>opentrust-observability</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>global/agents/observability-designer.md</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>opentrust-observability</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>devops-lead</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>OTAG24</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>incident-triage-specialist</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Triage incidents with smallest safe containment and recovery steps</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Incident phase, production/deployment issues</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Triage incidents, narrow blast radius, and propose recovery order.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>opentrust-observability</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>global/agents/incident-triage-specialist.md</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>opentrust-observability</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>devops-lead</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr"/>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>OTAG25</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>release-manager</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Gerenciar releases, changelog, versionamento semantico, depreciacao e notas de release</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Phase 5 (Ship), release planning and execution</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Plan, document and coordinate releases - semver, changelog, deprecation, release notes</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>opentrust-delivery; opentrust-observability</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>global/agents/release-manager.md</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>opentrust-delivery; opentrust-observability</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>delivery-lead</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr"/>
+      <c r="V52" t="inlineStr"/>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>Preserved legacy agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>OTAG26</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>changelog-writer</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Produces compact changelog entries from approved diffs and release facts</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Phase 5 (Ship), changelog generation</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Drafts changelog notes from approved scope, diff facts, and validation evidence.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>opentrust-delivery</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>global/agents/changelog-writer.md</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>opentrust-delivery</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>delivery-lead</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr"/>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>OTAG27</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>context-historian</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Tracks context lineage, decisions, and selector history across tasks</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>All phases, retrieval coherence tasks</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Tracks context decisions, selector use, and knowledge continuity across tasks.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>opentrust-reference-research; opentrust-observability</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>global/agents/context-historian.md</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>opentrust-reference-research; opentrust-observability</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>knowledge-lead</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr"/>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>OTAG28</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>reference-librarian</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Curates selector mappings, bundles, and reference profile consistency</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>All phases, selector/bundle curation</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Curates selector sets, bundle fit, and reference profile consistency.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>opentrust-reference-research</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>global/agents/reference-librarian.md</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>opentrust-reference-research</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>knowledge-lead</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>OTAG29</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>documentation-skill-creator</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Shapes documentation and skill drafts around approved selectors and source policy</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>All phases, doc/skill creation</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Prepares documentation and skill creation guidance from approved selectors and reference policy.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>opentrust-reference-research</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>global/agents/documentation-skill-creator.md</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>opentrust-reference-research</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>knowledge-lead</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>subagent</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>opentrust</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>opentrust-runtime</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr"/>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -50276,7 +54447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51326,6 +55497,102 @@
       <c r="H25" t="inlineStr">
         <is>
           <t>Monte uma estratégia de refeições para {objetivo}, com compras, preparo em lote, conservação, variedade e pontos de validação nutricional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>B25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>opentrust-workflow-core</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Core workflow contract, TDD, and spec-change for OpenTrust</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK02; OTSK03</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>OTLD01; OTLD02; OTLD03; OTLD04; OTLD05; OTLD08</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Explore &gt; Propose &gt; Apply phases. Use when: starting a new task, defining scope, planning implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>B26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>opentrust-delivery-core</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Review, delivery, and observability for OpenTrust</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OTSK04; OTSK05; OTSK06</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>OTLD06; OTLD07; OTLD08; OTLD09</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Review &gt; Ship phases. Use when: reviewing a diff, preparing release, logging decisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>B27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>opentrust-retrieval-core</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Reference research and retrieval governance for OpenTrust</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>OTSK07</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>OTLD09; OTAG27; OTAG28; OTAG29</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Any phase. Use when: domain knowledge is needed, task contract specifies selectors.</t>
         </is>
       </c>
     </row>
@@ -51340,7 +55607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52016,6 +56283,46 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>plano gradual; checklist; meal prep; perguntas para profissional; monitoramento</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PRJ13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>OpenStrut / OpenTrust</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Versioned engineering harness and runtime for OpenCode with OpenTrust topology</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK02; OTSK03; OTSK04; OTSK05; OTSK06; OTSK07</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>OTLD01; OTLD02; OTLD03; OTLD04; OTLD05; OTLD06; OTLD07; OTLD08; OTLD09</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>How to install? How to update agents? How to create a task contract? How to run a workflow?</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Installed runtime with 68 artifacts, 38 agents, 7 commands, 7 skills</t>
         </is>
       </c>
     </row>
@@ -52030,7 +56337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53205,6 +57512,280 @@
       <c r="I25" t="inlineStr">
         <is>
           <t>Decisão de curadoria com justificativa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>OpenTrust — iniciar workflow</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Iniciar um novo workflow OpenTrust: explorar, propor, implementar</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>OTLD01</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>OTSK01</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>B25</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>TEAM_TOPOLOGY.md; WORKFLOW.md; TASK_CONTRACT.md</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Objetivo: {objetivo}. Contexto: {contexto}. Siga o workflow OpenTrust: 1) Explore o estado atual, 2) Proponha um task contract com acceptance criteria e selectores de retrieval, 3) Obtenha aprovação antes de implementar.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Task contract aprovado, plano de execução, próximos passos</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>P26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>OpenTrust — revisar diff</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Revisar um diff de implementação antes do delivery</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OTLD06</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>OTSK04</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>B26</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>diff da implementação; task contract aprovado; resultados de teste</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Revisão do diff #{pr}. Verifique: 1) Acceptance criteria atendidos, 2) Cobertura de testes, 3) Segurança e privacidade, 4) Contratos e migrações, 5) Documentação. Aprova ou bloqueie com evidência.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Relatório de revisão com achados, aprovação ou bloqueios</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>P27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>OpenTrust — fazer release</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Preparar commit, push e PR para entrega</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>OTLD08</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>OTSK05</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>B26</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>diff final; relatório de revisão; resultados de validação</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Release {versao}: 1) Arquive documentação, 2) Commit com Conventional Commit, 3) Push, 4) Crie PR, 5) Tag e release. Use apenas arquivos aprovados.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Commit, push, PR criado, release publicado</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>P28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>OpenTrust — consultar referência</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Pesquisar material de referência usando selectores OpenTrust</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>OTLD09</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>OTSK07</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>B27</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>OPERATIONAL_RETRIEVAL_MAP.md; selectores CTX/SK/B/DOC</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Selectores: {selectores}. Contexto: {contexto}. Consulte o Operational Retrieval Map, peça síntese ao provider de retrieval. Retorne apenas síntese, sem chunks brutos. Inclua source IDs.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Síntese com source IDs, sem chunks brutos</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>P29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>OpenTrust — investigar incidente</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Triar e recuperar de incidente com evidência</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>OTLD07</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>OTSK06</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>logs; métricas; mudanças recentes; task contract ativo</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Incidente: {descricao}. 1) Diagnostique coletando evidência, 2) Contenha o dano, 3) Proponha recuperação, 4) Valide a resolução, 5) Reporte.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Diagnóstico, plano de contenção, recuperação validada, relatório</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>P30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>OpenTrust — verificar status</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Resumir estado atual do workflow e próximos passos</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>OTLD01</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>OTSK06</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>git status; diff; task plan ativo; últimas validações</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Resuma: branch, diff, tarefa ativa, fase do workflow, validações pendentes, próximo passo.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Resumo de estado com próximo passo claro</t>
         </is>
       </c>
     </row>
@@ -53219,7 +57800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54103,6 +58684,214 @@
       <c r="J17" t="inlineStr">
         <is>
           <t>Busque na documentação oficial de Odysseus a informação atual sobre {problema}, incluindo versão, exemplo mínimo e limitações.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DOC17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>OpenTrust Team Topology</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>opentrust/docs/TEAM_TOPOLOGY.md</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>9-team topology, workflow phases, and agent interaction model for OpenTrust</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK07</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>OTLD01; OTLD09</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>OpenStrut</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>When understanding team roles, workflow phases, or agent coordination</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Not for runtime or tool-specific questions</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Consulte a documentação de topologia OpenTrust para entender {dúvida}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DOC18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>OpenTrust Workflow</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>opentrust/docs/WORKFLOW.md</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Workflow phases, gates, retrieval rules, and transition checklist for OpenTrust</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK03; OTSK04</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>OTLD01; OTLD04; OTLD06</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OpenStrut</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>When planning or executing a workflow phase transition</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Not for agent-specific prompts or skill details</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Consulte o workflow OpenTrust para {fase} as regras de transição</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DOC19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>OpenTrust Task Contract</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>opentrust/docs/TASK_CONTRACT.md</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Task contract template with retrieval context, teams, and Definition of Done</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>OTSK01; OTSK03</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>OTLD01; OTLD02; OTLD03; OTLD04; OTLD08</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OpenStrut</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>When formalizing scope, AC, retrieval requirements, and delivery rules</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Not for informal or trivial tasks without retrieval needs</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Consulte o template de task contract para {tarefa}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DOC20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>OpenTrust Operational Retrieval Map</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>opentrust/docs/OPERATIONAL_RETRIEVAL_MAP.md</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Three-layer retrieval architecture: selectors, reference map, and provider policy</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>OTSK07</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>OTLD09; OTAG27; OTAG28</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OpenStrut</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>When understanding selector system, reference profiles, or retrieval policy</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Not for actual retrieval queries (use provider directly)</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Consulte o mapa de recuperação operacional para {seletor}</t>
         </is>
       </c>
     </row>

</xml_diff>